<commit_message>
cleaned up VWC analysis
</commit_message>
<xml_diff>
--- a/soilgrids_vs_field_statistics.xlsx
+++ b/soilgrids_vs_field_statistics.xlsx
@@ -588,19 +588,19 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>-0.15927</v>
+        <v>-0.15944</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>0.15927</v>
+        <v>0.15944</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0.16896</v>
+        <v>0.16931</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>51.81</v>
+        <v>51.91</v>
       </c>
       <c r="H4" s="2" t="n">
         <v>0</v>

</xml_diff>